<commit_message>
fix(analisis): etiquetas n (%) con total real, causas legibles en móvil y datos realistas cargables
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/pruebas/realista_mortalidad_550.xlsx
+++ b/data/pruebas/realista_mortalidad_550.xlsx
@@ -584,17 +584,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>21/05/1996</t>
+          <t>23/03/2004</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>IPS (centro/puesto salud)</t>
+          <t>Domicilio</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>23/07/2025</t>
+          <t>25/05/2026</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -640,7 +640,7 @@
         <v>4</v>
       </c>
       <c r="S2" t="n">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
@@ -654,7 +654,7 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>O15.0</t>
+          <t>O26.6</t>
         </is>
       </c>
       <c r="W2" t="n">
@@ -706,17 +706,17 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>05/01/2003</t>
+          <t>17/08/1984</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Lugar de trabajo</t>
+          <t>IPS (hospital/clínica)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>11/09/2025</t>
+          <t>23/04/2026</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -762,7 +762,7 @@
         <v>4</v>
       </c>
       <c r="S3" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="T3" t="inlineStr">
         <is>
@@ -776,7 +776,7 @@
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>O44.0</t>
+          <t>O26.6</t>
         </is>
       </c>
       <c r="W3" t="n">
@@ -793,22 +793,22 @@
       </c>
       <c r="AA3" t="inlineStr">
         <is>
-          <t>Urbana</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="AB3" t="inlineStr">
         <is>
-          <t>Desplazada</t>
+          <t>Ninguna</t>
         </is>
       </c>
       <c r="AC3" t="inlineStr">
         <is>
-          <t>Ninguna</t>
+          <t>Rrom</t>
         </is>
       </c>
       <c r="AD3" t="inlineStr">
         <is>
-          <t>Subsidiado</t>
+          <t>Contributivo</t>
         </is>
       </c>
     </row>
@@ -828,17 +828,17 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>21/08/1988</t>
+          <t>27/11/1987</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>IPS (centro/puesto salud)</t>
+          <t>Domicilio</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>04/05/2025</t>
+          <t>09/08/2026</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -884,7 +884,7 @@
         <v>1</v>
       </c>
       <c r="S4" t="n">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="T4" t="inlineStr">
         <is>
@@ -898,7 +898,7 @@
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>O41.1</t>
+          <t>O14.1</t>
         </is>
       </c>
       <c r="W4" t="n">
@@ -915,12 +915,12 @@
       </c>
       <c r="AA4" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Urbana</t>
         </is>
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>Ninguna</t>
+          <t>Desplazada</t>
         </is>
       </c>
       <c r="AC4" t="inlineStr">
@@ -930,7 +930,7 @@
       </c>
       <c r="AD4" t="inlineStr">
         <is>
-          <t>Contributivo</t>
+          <t>Subsidiado</t>
         </is>
       </c>
     </row>
@@ -950,17 +950,17 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>20/11/1993</t>
+          <t>29/03/1992</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Otro</t>
+          <t>Domicilio</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>15/02/2025</t>
+          <t>24/06/2025</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -1006,7 +1006,7 @@
         <v>4</v>
       </c>
       <c r="S5" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="T5" t="inlineStr">
         <is>
@@ -1020,7 +1020,7 @@
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>O44.0</t>
+          <t>O85</t>
         </is>
       </c>
       <c r="W5" t="n">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="AA5" t="inlineStr">
         <is>
-          <t>Urbana</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="AB5" t="inlineStr">
@@ -1072,17 +1072,17 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>07/11/2009</t>
+          <t>01/10/1997</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>IPS (hospital/clínica)</t>
+          <t>Domicilio</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>14/07/2026</t>
+          <t>07/06/2025</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -1128,7 +1128,7 @@
         <v>1</v>
       </c>
       <c r="S6" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="T6" t="inlineStr">
         <is>
@@ -1164,7 +1164,7 @@
       </c>
       <c r="AB6" t="inlineStr">
         <is>
-          <t>Ninguna</t>
+          <t>Desplazada</t>
         </is>
       </c>
       <c r="AC6" t="inlineStr">
@@ -1194,17 +1194,17 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>13/04/1992</t>
+          <t>10/03/1990</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Vía pública</t>
+          <t>IPS (hospital/clínica)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>02/10/2025</t>
+          <t>29/08/2026</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1250,7 +1250,7 @@
         <v>1</v>
       </c>
       <c r="S7" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="T7" t="inlineStr">
         <is>
@@ -1264,7 +1264,7 @@
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>O98.0</t>
+          <t>O14.1</t>
         </is>
       </c>
       <c r="W7" t="n">
@@ -1281,7 +1281,7 @@
       </c>
       <c r="AA7" t="inlineStr">
         <is>
-          <t>Urbana</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="AB7" t="inlineStr">
@@ -1296,7 +1296,7 @@
       </c>
       <c r="AD7" t="inlineStr">
         <is>
-          <t>Subsidiado</t>
+          <t>Contributivo</t>
         </is>
       </c>
     </row>
@@ -1316,17 +1316,17 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>16/03/2003</t>
+          <t>31/08/1987</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Otro</t>
+          <t>IPS (hospital/clínica)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>01/01/2026</t>
+          <t>17/06/2026</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1372,7 +1372,7 @@
         <v>3</v>
       </c>
       <c r="S8" t="n">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="T8" t="inlineStr">
         <is>
@@ -1408,7 +1408,7 @@
       </c>
       <c r="AB8" t="inlineStr">
         <is>
-          <t>Ninguna</t>
+          <t>Afro</t>
         </is>
       </c>
       <c r="AC8" t="inlineStr">
@@ -1438,17 +1438,17 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>27/09/1991</t>
+          <t>19/11/1991</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Otro</t>
+          <t>Domicilio</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>08/06/2025</t>
+          <t>31/07/2025</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1494,7 +1494,7 @@
         <v>1</v>
       </c>
       <c r="S9" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="T9" t="inlineStr">
         <is>
@@ -1508,7 +1508,7 @@
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>O85</t>
+          <t>O41.1</t>
         </is>
       </c>
       <c r="W9" t="n">
@@ -1525,22 +1525,22 @@
       </c>
       <c r="AA9" t="inlineStr">
         <is>
-          <t>Urbana</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="AB9" t="inlineStr">
         <is>
-          <t>Desplazada</t>
+          <t>Víctima de conflicto</t>
         </is>
       </c>
       <c r="AC9" t="inlineStr">
         <is>
-          <t>Afrocolombiana</t>
+          <t>Ninguna</t>
         </is>
       </c>
       <c r="AD9" t="inlineStr">
         <is>
-          <t>Contributivo</t>
+          <t>Subsidiado</t>
         </is>
       </c>
     </row>
@@ -1560,17 +1560,17 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>14/07/1983</t>
+          <t>26/09/1984</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Lugar de trabajo</t>
+          <t>IPS (hospital/clínica)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>06/01/2025</t>
+          <t>21/03/2026</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1616,7 +1616,7 @@
         <v>4</v>
       </c>
       <c r="S10" t="n">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="T10" t="inlineStr">
         <is>
@@ -1647,22 +1647,22 @@
       </c>
       <c r="AA10" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Urbana</t>
         </is>
       </c>
       <c r="AB10" t="inlineStr">
         <is>
-          <t>Ninguna</t>
+          <t>Víctima de conflicto</t>
         </is>
       </c>
       <c r="AC10" t="inlineStr">
         <is>
-          <t>Ninguna</t>
+          <t>Indígena</t>
         </is>
       </c>
       <c r="AD10" t="inlineStr">
         <is>
-          <t>Contributivo</t>
+          <t>Subsidiado</t>
         </is>
       </c>
     </row>
@@ -1682,7 +1682,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>15/05/2009</t>
+          <t>08/06/1998</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1692,7 +1692,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>17/11/2025</t>
+          <t>11/12/2025</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1738,7 +1738,7 @@
         <v>4</v>
       </c>
       <c r="S11" t="n">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="T11" t="inlineStr">
         <is>
@@ -1752,7 +1752,7 @@
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>O26.6</t>
+          <t>O14.1</t>
         </is>
       </c>
       <c r="W11" t="n">
@@ -1779,7 +1779,7 @@
       </c>
       <c r="AC11" t="inlineStr">
         <is>
-          <t>Ninguna</t>
+          <t>Afrocolombiana</t>
         </is>
       </c>
       <c r="AD11" t="inlineStr">
@@ -1804,17 +1804,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>03/11/1987</t>
+          <t>28/06/2007</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Lugar de trabajo</t>
+          <t>IPS (hospital/clínica)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>21/08/2026</t>
+          <t>15/04/2026</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1860,7 +1860,7 @@
         <v>1</v>
       </c>
       <c r="S12" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="T12" t="inlineStr">
         <is>
@@ -1874,7 +1874,7 @@
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>O99.3</t>
+          <t>O41.1</t>
         </is>
       </c>
       <c r="W12" t="n">
@@ -1896,17 +1896,17 @@
       </c>
       <c r="AB12" t="inlineStr">
         <is>
-          <t>Ninguna</t>
+          <t>Desplazada</t>
         </is>
       </c>
       <c r="AC12" t="inlineStr">
         <is>
-          <t>Ninguna</t>
+          <t>Raizal</t>
         </is>
       </c>
       <c r="AD12" t="inlineStr">
         <is>
-          <t>Subsidiado</t>
+          <t>Contributivo</t>
         </is>
       </c>
     </row>
@@ -1926,17 +1926,17 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>13/12/1992</t>
+          <t>28/12/1993</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>IPS (hospital/clínica)</t>
+          <t>Domicilio</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>12/08/2026</t>
+          <t>27/08/2025</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1982,7 +1982,7 @@
         <v>1</v>
       </c>
       <c r="S13" t="n">
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="T13" t="inlineStr">
         <is>
@@ -2018,17 +2018,17 @@
       </c>
       <c r="AB13" t="inlineStr">
         <is>
-          <t>Ninguna</t>
+          <t>Desplazada</t>
         </is>
       </c>
       <c r="AC13" t="inlineStr">
         <is>
-          <t>Ninguna</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="AD13" t="inlineStr">
         <is>
-          <t>Contributivo</t>
+          <t>Subsidiado</t>
         </is>
       </c>
     </row>
@@ -2048,17 +2048,17 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>07/09/1996</t>
+          <t>02/07/1993</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>IPS (centro/puesto salud)</t>
+          <t>IPS (hospital/clínica)</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>19/05/2026</t>
+          <t>13/03/2025</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -2104,7 +2104,7 @@
         <v>2</v>
       </c>
       <c r="S14" t="n">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="T14" t="inlineStr">
         <is>
@@ -2118,7 +2118,7 @@
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>O99.3</t>
+          <t>O15.0</t>
         </is>
       </c>
       <c r="W14" t="n">
@@ -2135,7 +2135,7 @@
       </c>
       <c r="AA14" t="inlineStr">
         <is>
-          <t>Urbana</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="AB14" t="inlineStr">
@@ -2170,17 +2170,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>04/10/1991</t>
+          <t>29/11/1994</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Lugar de trabajo</t>
+          <t>IPS (centro/puesto de salud)</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>19/05/2025</t>
+          <t>15/07/2026</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -2226,7 +2226,7 @@
         <v>4</v>
       </c>
       <c r="S15" t="n">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="T15" t="inlineStr">
         <is>
@@ -2240,7 +2240,7 @@
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>O85</t>
+          <t>O15.0</t>
         </is>
       </c>
       <c r="W15" t="n">
@@ -2257,12 +2257,12 @@
       </c>
       <c r="AA15" t="inlineStr">
         <is>
-          <t>Urbana</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="AB15" t="inlineStr">
         <is>
-          <t>Migrante</t>
+          <t>Indígena</t>
         </is>
       </c>
       <c r="AC15" t="inlineStr">
@@ -2272,7 +2272,7 @@
       </c>
       <c r="AD15" t="inlineStr">
         <is>
-          <t>Contributivo</t>
+          <t>Subsidiado</t>
         </is>
       </c>
     </row>
@@ -2292,17 +2292,17 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>11/12/2009</t>
+          <t>14/07/2007</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Otro</t>
+          <t>Domicilio</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>13/07/2026</t>
+          <t>13/02/2026</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -2348,7 +2348,7 @@
         <v>4</v>
       </c>
       <c r="S16" t="n">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="T16" t="inlineStr">
         <is>
@@ -2362,7 +2362,7 @@
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>O14.1</t>
+          <t>O98.0</t>
         </is>
       </c>
       <c r="W16" t="n">
@@ -2379,7 +2379,7 @@
       </c>
       <c r="AA16" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Urbana</t>
         </is>
       </c>
       <c r="AB16" t="inlineStr">
@@ -2394,7 +2394,7 @@
       </c>
       <c r="AD16" t="inlineStr">
         <is>
-          <t>Contributivo</t>
+          <t>Subsidiado</t>
         </is>
       </c>
     </row>
@@ -2414,17 +2414,17 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>12/06/1992</t>
+          <t>30/11/1988</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>IPS (centro/puesto salud)</t>
+          <t>Vía pública</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>17/08/2025</t>
+          <t>04/02/2025</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -2484,7 +2484,7 @@
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>O14.1</t>
+          <t>O85</t>
         </is>
       </c>
       <c r="W17" t="n">
@@ -2501,12 +2501,12 @@
       </c>
       <c r="AA17" t="inlineStr">
         <is>
-          <t>Urbana</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="AB17" t="inlineStr">
         <is>
-          <t>Migrante</t>
+          <t>Ninguna</t>
         </is>
       </c>
       <c r="AC17" t="inlineStr">
@@ -2516,7 +2516,7 @@
       </c>
       <c r="AD17" t="inlineStr">
         <is>
-          <t>Subsidiado</t>
+          <t>Contributivo</t>
         </is>
       </c>
     </row>
@@ -2536,17 +2536,17 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>17/04/2004</t>
+          <t>07/07/1994</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Domicilio</t>
+          <t>IPS (hospital/clínica)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>30/04/2026</t>
+          <t>20/07/2025</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -2592,7 +2592,7 @@
         <v>2</v>
       </c>
       <c r="S18" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="T18" t="inlineStr">
         <is>
@@ -2606,7 +2606,7 @@
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>O15.0</t>
+          <t>O14.1</t>
         </is>
       </c>
       <c r="W18" t="n">
@@ -2658,17 +2658,17 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>21/12/1987</t>
+          <t>21/10/1993</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Otro</t>
+          <t>IPS (hospital/clínica)</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>27/06/2025</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2714,7 +2714,7 @@
         <v>2</v>
       </c>
       <c r="S19" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T19" t="inlineStr">
         <is>
@@ -2728,7 +2728,7 @@
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>O14.1</t>
+          <t>O99.3</t>
         </is>
       </c>
       <c r="W19" t="n">
@@ -2745,7 +2745,7 @@
       </c>
       <c r="AA19" t="inlineStr">
         <is>
-          <t>Urbana</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="AB19" t="inlineStr">
@@ -2760,7 +2760,7 @@
       </c>
       <c r="AD19" t="inlineStr">
         <is>
-          <t>Subsidiado</t>
+          <t>Contributivo</t>
         </is>
       </c>
     </row>
@@ -2780,17 +2780,17 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>03/08/1986</t>
+          <t>07/05/2002</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>IPS (centro/puesto salud)</t>
+          <t>IPS (centro/puesto de salud)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>15/05/2025</t>
+          <t>16/02/2025</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -2836,7 +2836,7 @@
         <v>1</v>
       </c>
       <c r="S20" t="n">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="T20" t="inlineStr">
         <is>
@@ -2850,7 +2850,7 @@
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>O14.1</t>
+          <t>O15.0</t>
         </is>
       </c>
       <c r="W20" t="n">
@@ -2867,12 +2867,12 @@
       </c>
       <c r="AA20" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Urbana</t>
         </is>
       </c>
       <c r="AB20" t="inlineStr">
         <is>
-          <t>Migrante</t>
+          <t>Ninguna</t>
         </is>
       </c>
       <c r="AC20" t="inlineStr">
@@ -2882,7 +2882,7 @@
       </c>
       <c r="AD20" t="inlineStr">
         <is>
-          <t>Contributivo</t>
+          <t>No afiliada</t>
         </is>
       </c>
     </row>
@@ -2902,17 +2902,17 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>11/03/2008</t>
+          <t>21/04/2001</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Otro</t>
+          <t>IPS (hospital/clínica)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>01/06/2026</t>
+          <t>12/07/2026</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2958,7 +2958,7 @@
         <v>4</v>
       </c>
       <c r="S21" t="n">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="T21" t="inlineStr">
         <is>
@@ -2972,7 +2972,7 @@
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>O98.0</t>
+          <t>O15.0</t>
         </is>
       </c>
       <c r="W21" t="n">
@@ -2989,7 +2989,7 @@
       </c>
       <c r="AA21" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Urbana</t>
         </is>
       </c>
       <c r="AB21" t="inlineStr">
@@ -2999,12 +2999,12 @@
       </c>
       <c r="AC21" t="inlineStr">
         <is>
-          <t>Indígena</t>
+          <t>Afrocolombiana</t>
         </is>
       </c>
       <c r="AD21" t="inlineStr">
         <is>
-          <t>Contributivo</t>
+          <t>Subsidiado</t>
         </is>
       </c>
     </row>
@@ -3024,7 +3024,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>12/03/1992</t>
+          <t>07/07/1999</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -3034,7 +3034,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>25/10/2025</t>
+          <t>19/02/2025</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -3080,7 +3080,7 @@
         <v>1</v>
       </c>
       <c r="S22" t="n">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="T22" t="inlineStr">
         <is>
@@ -3094,7 +3094,7 @@
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>O85</t>
+          <t>O14.1</t>
         </is>
       </c>
       <c r="W22" t="n">
@@ -3116,7 +3116,7 @@
       </c>
       <c r="AB22" t="inlineStr">
         <is>
-          <t>Ninguna</t>
+          <t>Migrante</t>
         </is>
       </c>
       <c r="AC22" t="inlineStr">
@@ -3126,7 +3126,7 @@
       </c>
       <c r="AD22" t="inlineStr">
         <is>
-          <t>Subsidiado</t>
+          <t>Contributivo</t>
         </is>
       </c>
     </row>
@@ -3146,17 +3146,17 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>06/11/2002</t>
+          <t>17/11/1994</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Durante traslado</t>
+          <t>Durante el traslado</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>28/03/2025</t>
+          <t>08/04/2026</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -3202,7 +3202,7 @@
         <v>3</v>
       </c>
       <c r="S23" t="n">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="T23" t="inlineStr">
         <is>
@@ -3216,7 +3216,7 @@
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>O15.0</t>
+          <t>O14.1</t>
         </is>
       </c>
       <c r="W23" t="n">
@@ -3238,7 +3238,7 @@
       </c>
       <c r="AB23" t="inlineStr">
         <is>
-          <t>Discapacidad</t>
+          <t>Ninguna</t>
         </is>
       </c>
       <c r="AC23" t="inlineStr">
@@ -3248,7 +3248,7 @@
       </c>
       <c r="AD23" t="inlineStr">
         <is>
-          <t>Subsidiado</t>
+          <t>Contributivo</t>
         </is>
       </c>
     </row>
@@ -3268,17 +3268,17 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>07/10/2000</t>
+          <t>15/02/2007</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>IPS (centro/puesto salud)</t>
+          <t>Domicilio</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>04/03/2026</t>
+          <t>13/07/2025</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -3324,7 +3324,7 @@
         <v>3</v>
       </c>
       <c r="S24" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="T24" t="inlineStr">
         <is>
@@ -3338,7 +3338,7 @@
       </c>
       <c r="V24" t="inlineStr">
         <is>
-          <t>O85</t>
+          <t>O44.0</t>
         </is>
       </c>
       <c r="W24" t="n">
@@ -3360,7 +3360,7 @@
       </c>
       <c r="AB24" t="inlineStr">
         <is>
-          <t>Migrante</t>
+          <t>Ninguna</t>
         </is>
       </c>
       <c r="AC24" t="inlineStr">
@@ -3370,7 +3370,7 @@
       </c>
       <c r="AD24" t="inlineStr">
         <is>
-          <t>Contributivo</t>
+          <t>Subsidiado</t>
         </is>
       </c>
     </row>
@@ -3390,17 +3390,17 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>01/04/1994</t>
+          <t>27/02/2001</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Vía pública</t>
+          <t>IPS (hospital/clínica)</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>13/06/2025</t>
+          <t>11/05/2026</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -3446,7 +3446,7 @@
         <v>1</v>
       </c>
       <c r="S25" t="n">
-        <v>27</v>
+        <v>39</v>
       </c>
       <c r="T25" t="inlineStr">
         <is>
@@ -3512,17 +3512,17 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>19/10/1986</t>
+          <t>23/06/1983</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Otro</t>
+          <t>IPS (centro/puesto de salud)</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>19/05/2025</t>
+          <t>21/01/2025</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -3568,7 +3568,7 @@
         <v>4</v>
       </c>
       <c r="S26" t="n">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="T26" t="inlineStr">
         <is>
@@ -3582,7 +3582,7 @@
       </c>
       <c r="V26" t="inlineStr">
         <is>
-          <t>O44.0</t>
+          <t>O85</t>
         </is>
       </c>
       <c r="W26" t="n">
@@ -3614,7 +3614,7 @@
       </c>
       <c r="AD26" t="inlineStr">
         <is>
-          <t>No afiliada</t>
+          <t>Contributivo</t>
         </is>
       </c>
     </row>
@@ -3634,17 +3634,17 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>09/06/1999</t>
+          <t>26/02/2003</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>IPS (centro/puesto salud)</t>
+          <t>IPS (hospital/clínica)</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>24/08/2026</t>
+          <t>13/05/2025</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -3690,7 +3690,7 @@
         <v>4</v>
       </c>
       <c r="S27" t="n">
-        <v>41</v>
+        <v>20</v>
       </c>
       <c r="T27" t="inlineStr">
         <is>
@@ -3704,7 +3704,7 @@
       </c>
       <c r="V27" t="inlineStr">
         <is>
-          <t>O15.0</t>
+          <t>O85</t>
         </is>
       </c>
       <c r="W27" t="n">
@@ -3726,12 +3726,12 @@
       </c>
       <c r="AB27" t="inlineStr">
         <is>
-          <t>Ninguna</t>
+          <t>Discapacidad</t>
         </is>
       </c>
       <c r="AC27" t="inlineStr">
         <is>
-          <t>Rrom</t>
+          <t>Ninguna</t>
         </is>
       </c>
       <c r="AD27" t="inlineStr">
@@ -3756,17 +3756,17 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>25/03/2003</t>
+          <t>09/11/1992</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Lugar de trabajo</t>
+          <t>IPS (centro/puesto de salud)</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>10/11/2025</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -3812,7 +3812,7 @@
         <v>3</v>
       </c>
       <c r="S28" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="T28" t="inlineStr">
         <is>
@@ -3826,7 +3826,7 @@
       </c>
       <c r="V28" t="inlineStr">
         <is>
-          <t>O15.0</t>
+          <t>O85</t>
         </is>
       </c>
       <c r="W28" t="n">
@@ -3848,12 +3848,12 @@
       </c>
       <c r="AB28" t="inlineStr">
         <is>
-          <t>Ninguna</t>
+          <t>Desplazada</t>
         </is>
       </c>
       <c r="AC28" t="inlineStr">
         <is>
-          <t>Indígena</t>
+          <t>Ninguna</t>
         </is>
       </c>
       <c r="AD28" t="inlineStr">
@@ -3878,17 +3878,17 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>03/11/2003</t>
+          <t>10/01/1989</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Lugar de trabajo</t>
+          <t>Vía pública</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>04/06/2026</t>
+          <t>12/08/2025</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -3934,7 +3934,7 @@
         <v>4</v>
       </c>
       <c r="S29" t="n">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="T29" t="inlineStr">
         <is>
@@ -3948,7 +3948,7 @@
       </c>
       <c r="V29" t="inlineStr">
         <is>
-          <t>O99.3</t>
+          <t>O26.6</t>
         </is>
       </c>
       <c r="W29" t="n">
@@ -3965,12 +3965,12 @@
       </c>
       <c r="AA29" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Urbana</t>
         </is>
       </c>
       <c r="AB29" t="inlineStr">
         <is>
-          <t>Desplazada</t>
+          <t>Indígena</t>
         </is>
       </c>
       <c r="AC29" t="inlineStr">
@@ -4000,17 +4000,17 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>07/12/1996</t>
+          <t>25/03/1990</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>IPS (hospital/clínica)</t>
+          <t>Lugar de trabajo</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>26/02/2026</t>
+          <t>14/06/2026</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -4056,7 +4056,7 @@
         <v>3</v>
       </c>
       <c r="S30" t="n">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="T30" t="inlineStr">
         <is>
@@ -4070,7 +4070,7 @@
       </c>
       <c r="V30" t="inlineStr">
         <is>
-          <t>O08.1</t>
+          <t>O14.1</t>
         </is>
       </c>
       <c r="W30" t="n">
@@ -4087,17 +4087,17 @@
       </c>
       <c r="AA30" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Urbana</t>
         </is>
       </c>
       <c r="AB30" t="inlineStr">
         <is>
-          <t>Ninguna</t>
+          <t>Indígena</t>
         </is>
       </c>
       <c r="AC30" t="inlineStr">
         <is>
-          <t>Afrocolombiana</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="AD30" t="inlineStr">
@@ -4122,17 +4122,17 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>18/11/1984</t>
+          <t>05/03/2003</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>IPS (centro/puesto salud)</t>
+          <t>IPS (hospital/clínica)</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>04/02/2026</t>
+          <t>22/05/2025</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -4178,7 +4178,7 @@
         <v>2</v>
       </c>
       <c r="S31" t="n">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="T31" t="inlineStr">
         <is>
@@ -4192,7 +4192,7 @@
       </c>
       <c r="V31" t="inlineStr">
         <is>
-          <t>O41.1</t>
+          <t>O14.1</t>
         </is>
       </c>
       <c r="W31" t="n">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="AB31" t="inlineStr">
         <is>
-          <t>Ninguna</t>
+          <t>Migrante</t>
         </is>
       </c>
       <c r="AC31" t="inlineStr">
@@ -4224,7 +4224,7 @@
       </c>
       <c r="AD31" t="inlineStr">
         <is>
-          <t>Contributivo</t>
+          <t>Subsidiado</t>
         </is>
       </c>
     </row>
@@ -4244,17 +4244,17 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>18/05/1987</t>
+          <t>30/05/1992</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Domicilio</t>
+          <t>IPS (hospital/clínica)</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>02/06/2025</t>
+          <t>14/06/2025</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -4336,12 +4336,12 @@
       </c>
       <c r="AB32" t="inlineStr">
         <is>
-          <t>Ninguna</t>
+          <t>Migrante</t>
         </is>
       </c>
       <c r="AC32" t="inlineStr">
         <is>
-          <t>Ninguna</t>
+          <t>Afrocolombiana</t>
         </is>
       </c>
       <c r="AD32" t="inlineStr">
@@ -4366,7 +4366,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>30/04/2001</t>
+          <t>23/05/1996</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -4376,7 +4376,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>17/06/2026</t>
+          <t>10/07/2025</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -4422,7 +4422,7 @@
         <v>3</v>
       </c>
       <c r="S33" t="n">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="T33" t="inlineStr">
         <is>
@@ -4436,7 +4436,7 @@
       </c>
       <c r="V33" t="inlineStr">
         <is>
-          <t>O08.1</t>
+          <t>O14.1</t>
         </is>
       </c>
       <c r="W33" t="n">
@@ -4488,17 +4488,17 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>23/06/2003</t>
+          <t>07/01/2001</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Domicilio</t>
+          <t>IPS (hospital/clínica)</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>04/02/2026</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -4544,7 +4544,7 @@
         <v>4</v>
       </c>
       <c r="S34" t="n">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="T34" t="inlineStr">
         <is>
@@ -4558,7 +4558,7 @@
       </c>
       <c r="V34" t="inlineStr">
         <is>
-          <t>O15.0</t>
+          <t>O44.0</t>
         </is>
       </c>
       <c r="W34" t="n">
@@ -4590,7 +4590,7 @@
       </c>
       <c r="AD34" t="inlineStr">
         <is>
-          <t>Contributivo</t>
+          <t>No afiliada</t>
         </is>
       </c>
     </row>
@@ -4610,17 +4610,17 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>26/12/1994</t>
+          <t>11/09/1987</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Otro</t>
+          <t>IPS (hospital/clínica)</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>21/01/2026</t>
+          <t>07/10/2025</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -4680,7 +4680,7 @@
       </c>
       <c r="V35" t="inlineStr">
         <is>
-          <t>O14.1</t>
+          <t>O99.3</t>
         </is>
       </c>
       <c r="W35" t="n">
@@ -4702,7 +4702,7 @@
       </c>
       <c r="AB35" t="inlineStr">
         <is>
-          <t>Afro</t>
+          <t>Ninguna</t>
         </is>
       </c>
       <c r="AC35" t="inlineStr">
@@ -4732,17 +4732,17 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>08/01/1996</t>
+          <t>05/03/2001</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Durante traslado</t>
+          <t>IPS (hospital/clínica)</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>15/01/2025</t>
+          <t>12/03/2026</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -4788,7 +4788,7 @@
         <v>1</v>
       </c>
       <c r="S36" t="n">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="T36" t="inlineStr">
         <is>
@@ -4802,7 +4802,7 @@
       </c>
       <c r="V36" t="inlineStr">
         <is>
-          <t>O41.1</t>
+          <t>O94</t>
         </is>
       </c>
       <c r="W36" t="n">
@@ -4824,7 +4824,7 @@
       </c>
       <c r="AB36" t="inlineStr">
         <is>
-          <t>Indígena</t>
+          <t>Migrante</t>
         </is>
       </c>
       <c r="AC36" t="inlineStr">
@@ -4854,17 +4854,17 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>31/12/1993</t>
+          <t>13/03/2001</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Durante traslado</t>
+          <t>Domicilio</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>19/04/2025</t>
+          <t>30/06/2026</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -4910,7 +4910,7 @@
         <v>1</v>
       </c>
       <c r="S37" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T37" t="inlineStr">
         <is>
@@ -4924,7 +4924,7 @@
       </c>
       <c r="V37" t="inlineStr">
         <is>
-          <t>O41.1</t>
+          <t>O99.3</t>
         </is>
       </c>
       <c r="W37" t="n">
@@ -4946,7 +4946,7 @@
       </c>
       <c r="AB37" t="inlineStr">
         <is>
-          <t>Indígena</t>
+          <t>Ninguna</t>
         </is>
       </c>
       <c r="AC37" t="inlineStr">
@@ -4956,7 +4956,7 @@
       </c>
       <c r="AD37" t="inlineStr">
         <is>
-          <t>Subsidiado</t>
+          <t>Contributivo</t>
         </is>
       </c>
     </row>
@@ -4976,17 +4976,17 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>24/10/1994</t>
+          <t>19/11/2000</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Domicilio</t>
+          <t>IPS (hospital/clínica)</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>03/02/2026</t>
+          <t>01/03/2026</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -5032,7 +5032,7 @@
         <v>3</v>
       </c>
       <c r="S38" t="n">
-        <v>21</v>
+        <v>38</v>
       </c>
       <c r="T38" t="inlineStr">
         <is>
@@ -5046,7 +5046,7 @@
       </c>
       <c r="V38" t="inlineStr">
         <is>
-          <t>O15.0</t>
+          <t>O94</t>
         </is>
       </c>
       <c r="W38" t="n">
@@ -5068,12 +5068,12 @@
       </c>
       <c r="AB38" t="inlineStr">
         <is>
-          <t>Ninguna</t>
+          <t>Migrante</t>
         </is>
       </c>
       <c r="AC38" t="inlineStr">
         <is>
-          <t>Ninguna</t>
+          <t>Afrocolombiana</t>
         </is>
       </c>
       <c r="AD38" t="inlineStr">
@@ -5098,7 +5098,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>02/02/2000</t>
+          <t>07/02/2008</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -5108,7 +5108,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>17/03/2025</t>
+          <t>22/03/2025</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -5168,7 +5168,7 @@
       </c>
       <c r="V39" t="inlineStr">
         <is>
-          <t>O26.6</t>
+          <t>O15.0</t>
         </is>
       </c>
       <c r="W39" t="n">
@@ -5190,12 +5190,12 @@
       </c>
       <c r="AB39" t="inlineStr">
         <is>
-          <t>Ninguna</t>
+          <t>Desplazada</t>
         </is>
       </c>
       <c r="AC39" t="inlineStr">
         <is>
-          <t>Afrocolombiana</t>
+          <t>Ninguna</t>
         </is>
       </c>
       <c r="AD39" t="inlineStr">
@@ -5220,17 +5220,17 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>26/05/2007</t>
+          <t>01/05/1998</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Lugar de trabajo</t>
+          <t>Domicilio</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>22/02/2025</t>
+          <t>28/01/2026</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -5276,7 +5276,7 @@
         <v>2</v>
       </c>
       <c r="S40" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="T40" t="inlineStr">
         <is>
@@ -5290,7 +5290,7 @@
       </c>
       <c r="V40" t="inlineStr">
         <is>
-          <t>O15.0</t>
+          <t>O14.1</t>
         </is>
       </c>
       <c r="W40" t="n">
@@ -5312,7 +5312,7 @@
       </c>
       <c r="AB40" t="inlineStr">
         <is>
-          <t>Migrante</t>
+          <t>Ninguna</t>
         </is>
       </c>
       <c r="AC40" t="inlineStr">
@@ -5342,7 +5342,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>03/11/2003</t>
+          <t>21/09/1987</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -5352,7 +5352,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>22/12/2025</t>
+          <t>09/11/2025</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -5398,7 +5398,7 @@
         <v>1</v>
       </c>
       <c r="S41" t="n">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="T41" t="inlineStr">
         <is>
@@ -5412,7 +5412,7 @@
       </c>
       <c r="V41" t="inlineStr">
         <is>
-          <t>O85</t>
+          <t>O14.1</t>
         </is>
       </c>
       <c r="W41" t="n">
@@ -5429,7 +5429,7 @@
       </c>
       <c r="AA41" t="inlineStr">
         <is>
-          <t>Urbana</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="AB41" t="inlineStr">
@@ -5439,7 +5439,7 @@
       </c>
       <c r="AC41" t="inlineStr">
         <is>
-          <t>Ninguna</t>
+          <t>Indígena</t>
         </is>
       </c>
       <c r="AD41" t="inlineStr">
@@ -5464,7 +5464,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>28/12/2009</t>
+          <t>11/07/1989</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -5474,7 +5474,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>28/12/2025</t>
+          <t>11/07/2025</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -5520,7 +5520,7 @@
         <v>1</v>
       </c>
       <c r="S42" t="n">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="T42" t="inlineStr">
         <is>
@@ -5534,7 +5534,7 @@
       </c>
       <c r="V42" t="inlineStr">
         <is>
-          <t>O14.1</t>
+          <t>O98.0</t>
         </is>
       </c>
       <c r="W42" t="n">
@@ -5566,7 +5566,7 @@
       </c>
       <c r="AD42" t="inlineStr">
         <is>
-          <t>Subsidiado</t>
+          <t>Contributivo</t>
         </is>
       </c>
     </row>
@@ -5586,17 +5586,17 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>01/12/2007</t>
+          <t>23/10/1998</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>IPS (centro/puesto salud)</t>
+          <t>Durante el traslado</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>27/01/2025</t>
+          <t>19/12/2025</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -5642,7 +5642,7 @@
         <v>2</v>
       </c>
       <c r="S43" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="T43" t="inlineStr">
         <is>
@@ -5656,7 +5656,7 @@
       </c>
       <c r="V43" t="inlineStr">
         <is>
-          <t>O98.0</t>
+          <t>O14.1</t>
         </is>
       </c>
       <c r="W43" t="n">
@@ -5708,17 +5708,17 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>13/07/1995</t>
+          <t>12/12/2008</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Durante traslado</t>
+          <t>Vía pública</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>27/01/2025</t>
+          <t>28/06/2025</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -5764,7 +5764,7 @@
         <v>3</v>
       </c>
       <c r="S44" t="n">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="T44" t="inlineStr">
         <is>
@@ -5778,7 +5778,7 @@
       </c>
       <c r="V44" t="inlineStr">
         <is>
-          <t>O08.1</t>
+          <t>O15.0</t>
         </is>
       </c>
       <c r="W44" t="n">
@@ -5795,7 +5795,7 @@
       </c>
       <c r="AA44" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Urbana</t>
         </is>
       </c>
       <c r="AB44" t="inlineStr">
@@ -5805,7 +5805,7 @@
       </c>
       <c r="AC44" t="inlineStr">
         <is>
-          <t>Raizal</t>
+          <t>Ninguna</t>
         </is>
       </c>
       <c r="AD44" t="inlineStr">
@@ -5830,17 +5830,17 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>12/04/1999</t>
+          <t>02/08/2008</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Otro</t>
+          <t>Domicilio</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>07/06/2026</t>
+          <t>27/09/2025</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -5886,7 +5886,7 @@
         <v>2</v>
       </c>
       <c r="S45" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="T45" t="inlineStr">
         <is>
@@ -5900,7 +5900,7 @@
       </c>
       <c r="V45" t="inlineStr">
         <is>
-          <t>O98.0</t>
+          <t>O85</t>
         </is>
       </c>
       <c r="W45" t="n">
@@ -5922,7 +5922,7 @@
       </c>
       <c r="AB45" t="inlineStr">
         <is>
-          <t>Ninguna</t>
+          <t>Desplazada</t>
         </is>
       </c>
       <c r="AC45" t="inlineStr">
@@ -5932,7 +5932,7 @@
       </c>
       <c r="AD45" t="inlineStr">
         <is>
-          <t>Subsidiado</t>
+          <t>Contributivo</t>
         </is>
       </c>
     </row>
@@ -5952,17 +5952,17 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>15/11/1994</t>
+          <t>03/11/2009</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Domicilio</t>
+          <t>Durante el traslado</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>03/05/2026</t>
+          <t>21/04/2026</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -6008,7 +6008,7 @@
         <v>4</v>
       </c>
       <c r="S46" t="n">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="T46" t="inlineStr">
         <is>
@@ -6022,7 +6022,7 @@
       </c>
       <c r="V46" t="inlineStr">
         <is>
-          <t>O85</t>
+          <t>O08.1</t>
         </is>
       </c>
       <c r="W46" t="n">
@@ -6049,7 +6049,7 @@
       </c>
       <c r="AC46" t="inlineStr">
         <is>
-          <t>Indígena</t>
+          <t>Ninguna</t>
         </is>
       </c>
       <c r="AD46" t="inlineStr">
@@ -6074,17 +6074,17 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>13/02/1987</t>
+          <t>07/08/2007</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Vía pública</t>
+          <t>IPS (hospital/clínica)</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>02/12/2025</t>
+          <t>25/05/2026</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -6130,7 +6130,7 @@
         <v>4</v>
       </c>
       <c r="S47" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="T47" t="inlineStr">
         <is>
@@ -6144,7 +6144,7 @@
       </c>
       <c r="V47" t="inlineStr">
         <is>
-          <t>O26.6</t>
+          <t>O08.1</t>
         </is>
       </c>
       <c r="W47" t="n">
@@ -6161,12 +6161,12 @@
       </c>
       <c r="AA47" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Urbana</t>
         </is>
       </c>
       <c r="AB47" t="inlineStr">
         <is>
-          <t>Ninguna</t>
+          <t>Desplazada</t>
         </is>
       </c>
       <c r="AC47" t="inlineStr">
@@ -6196,17 +6196,17 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>03/05/1987</t>
+          <t>26/08/1992</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Domicilio</t>
+          <t>IPS (hospital/clínica)</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>07/11/2025</t>
+          <t>02/03/2026</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -6252,7 +6252,7 @@
         <v>3</v>
       </c>
       <c r="S48" t="n">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="T48" t="inlineStr">
         <is>
@@ -6266,7 +6266,7 @@
       </c>
       <c r="V48" t="inlineStr">
         <is>
-          <t>O98.0</t>
+          <t>O99.3</t>
         </is>
       </c>
       <c r="W48" t="n">
@@ -6293,7 +6293,7 @@
       </c>
       <c r="AC48" t="inlineStr">
         <is>
-          <t>Afrocolombiana</t>
+          <t>Ninguna</t>
         </is>
       </c>
       <c r="AD48" t="inlineStr">
@@ -6318,17 +6318,17 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>26/10/2003</t>
+          <t>12/05/1994</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Durante traslado</t>
+          <t>IPS (hospital/clínica)</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>06/04/2026</t>
+          <t>22/10/2025</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -6374,7 +6374,7 @@
         <v>3</v>
       </c>
       <c r="S49" t="n">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="T49" t="inlineStr">
         <is>
@@ -6388,7 +6388,7 @@
       </c>
       <c r="V49" t="inlineStr">
         <is>
-          <t>O98.0</t>
+          <t>O26.6</t>
         </is>
       </c>
       <c r="W49" t="n">
@@ -6410,7 +6410,7 @@
       </c>
       <c r="AB49" t="inlineStr">
         <is>
-          <t>Migrante</t>
+          <t>Ninguna</t>
         </is>
       </c>
       <c r="AC49" t="inlineStr">
@@ -6440,17 +6440,17 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>12/10/2009</t>
+          <t>06/03/1985</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Vía pública</t>
+          <t>IPS (hospital/clínica)</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>30/11/2025</t>
+          <t>24/04/2026</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -6510,7 +6510,7 @@
       </c>
       <c r="V50" t="inlineStr">
         <is>
-          <t>O85</t>
+          <t>O08.1</t>
         </is>
       </c>
       <c r="W50" t="n">
@@ -6527,12 +6527,12 @@
       </c>
       <c r="AA50" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Urbana</t>
         </is>
       </c>
       <c r="AB50" t="inlineStr">
         <is>
-          <t>Discapacidad</t>
+          <t>Ninguna</t>
         </is>
       </c>
       <c r="AC50" t="inlineStr">
@@ -6562,17 +6562,17 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>10/09/1986</t>
+          <t>06/11/1997</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>IPS (hospital/clínica)</t>
+          <t>IPS (centro/puesto de salud)</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>05/05/2025</t>
+          <t>01/07/2025</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -6618,7 +6618,7 @@
         <v>2</v>
       </c>
       <c r="S51" t="n">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="T51" t="inlineStr">
         <is>
@@ -6632,7 +6632,7 @@
       </c>
       <c r="V51" t="inlineStr">
         <is>
-          <t>O08.1</t>
+          <t>O85</t>
         </is>
       </c>
       <c r="W51" t="n">
@@ -6649,12 +6649,12 @@
       </c>
       <c r="AA51" t="inlineStr">
         <is>
-          <t>Urbana</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="AB51" t="inlineStr">
         <is>
-          <t>Migrante</t>
+          <t>Ninguna</t>
         </is>
       </c>
       <c r="AC51" t="inlineStr">
@@ -6664,7 +6664,7 @@
       </c>
       <c r="AD51" t="inlineStr">
         <is>
-          <t>Subsidiado</t>
+          <t>Contributivo</t>
         </is>
       </c>
     </row>
@@ -6684,17 +6684,17 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>10/08/1998</t>
+          <t>15/02/1989</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Domicilio</t>
+          <t>IPS (hospital/clínica)</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>25/05/2026</t>
+          <t>30/11/2025</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -6740,7 +6740,7 @@
         <v>4</v>
       </c>
       <c r="S52" t="n">
-        <v>41</v>
+        <v>23</v>
       </c>
       <c r="T52" t="inlineStr">
         <is>
@@ -6754,7 +6754,7 @@
       </c>
       <c r="V52" t="inlineStr">
         <is>
-          <t>O26.6</t>
+          <t>O08.1</t>
         </is>
       </c>
       <c r="W52" t="n">
@@ -6781,7 +6781,7 @@
       </c>
       <c r="AC52" t="inlineStr">
         <is>
-          <t>Afrocolombiana</t>
+          <t>Ninguna</t>
         </is>
       </c>
       <c r="AD52" t="inlineStr">
@@ -6806,17 +6806,17 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>04/07/1992</t>
+          <t>27/08/1992</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>IPS (centro/puesto salud)</t>
+          <t>IPS (hospital/clínica)</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>23/04/2026</t>
+          <t>16/06/2026</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -6862,7 +6862,7 @@
         <v>1</v>
       </c>
       <c r="S53" t="n">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="T53" t="inlineStr">
         <is>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="V53" t="inlineStr">
         <is>
-          <t>O08.1</t>
+          <t>O41.1</t>
         </is>
       </c>
       <c r="W53" t="n">
@@ -6928,17 +6928,17 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>19/12/1989</t>
+          <t>18/09/1992</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Otro</t>
+          <t>IPS (hospital/clínica)</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>09/08/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -6984,7 +6984,7 @@
         <v>3</v>
       </c>
       <c r="S54" t="n">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="T54" t="inlineStr">
         <is>
@@ -6998,7 +6998,7 @@
       </c>
       <c r="V54" t="inlineStr">
         <is>
-          <t>O44.0</t>
+          <t>O41.1</t>
         </is>
       </c>
       <c r="W54" t="n">
@@ -7015,7 +7015,7 @@
       </c>
       <c r="AA54" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Urbana</t>
         </is>
       </c>
       <c r="AB54" t="inlineStr">
@@ -7050,17 +7050,17 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>13/09/2002</t>
+          <t>21/06/1992</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Domicilio</t>
+          <t>IPS (hospital/clínica)</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>24/06/2025</t>
+          <t>01/04/2026</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -7106,7 +7106,7 @@
         <v>4</v>
       </c>
       <c r="S55" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="T55" t="inlineStr">
         <is>
@@ -7120,7 +7120,7 @@
       </c>
       <c r="V55" t="inlineStr">
         <is>
-          <t>O85</t>
+          <t>O14.1</t>
         </is>
       </c>
       <c r="W55" t="n">
@@ -7137,7 +7137,7 @@
       </c>
       <c r="AA55" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Urbana</t>
         </is>
       </c>
       <c r="AB55" t="inlineStr">
@@ -7147,7 +7147,7 @@
       </c>
       <c r="AC55" t="inlineStr">
         <is>
-          <t>Ninguna</t>
+          <t>Afrocolombiana</t>
         </is>
       </c>
       <c r="AD55" t="inlineStr">
@@ -7172,17 +7172,17 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>23/03/1992</t>
+          <t>17/02/1984</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Domicilio</t>
+          <t>IPS (hospital/clínica)</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>07/06/2025</t>
+          <t>03/05/2025</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -7228,7 +7228,7 @@
         <v>2</v>
       </c>
       <c r="S56" t="n">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="T56" t="inlineStr">
         <is>
@@ -7242,7 +7242,7 @@
       </c>
       <c r="V56" t="inlineStr">
         <is>
-          <t>O26.6</t>
+          <t>O14.1</t>
         </is>
       </c>
       <c r="W56" t="n">
@@ -7259,12 +7259,12 @@
       </c>
       <c r="AA56" t="inlineStr">
         <is>
-          <t>Urbana</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="AB56" t="inlineStr">
         <is>
-          <t>Afro</t>
+          <t>Ninguna</t>
         </is>
       </c>
       <c r="AC56" t="inlineStr">
@@ -7294,17 +7294,17 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>29/01/2001</t>
+          <t>24/11/2000</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Domicilio</t>
+          <t>IPS (hospital/clínica)</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>29/08/2026</t>
+          <t>24/06/2026</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -7350,7 +7350,7 @@
         <v>3</v>
       </c>
       <c r="S57" t="n">
-        <v>41</v>
+        <v>21</v>
       </c>
       <c r="T57" t="inlineStr">
         <is>
@@ -7364,7 +7364,7 @@
       </c>
       <c r="V57" t="inlineStr">
         <is>
-          <t>O08.1</t>
+          <t>O94</t>
         </is>
       </c>
       <c r="W57" t="n">
@@ -7391,12 +7391,12 @@
       </c>
       <c r="AC57" t="inlineStr">
         <is>
-          <t>Ninguna</t>
+          <t>Indígena</t>
         </is>
       </c>
       <c r="AD57" t="inlineStr">
         <is>
-          <t>Subsidiado</t>
+          <t>Contributivo</t>
         </is>
       </c>
     </row>
@@ -7416,17 +7416,17 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>25/11/1989</t>
+          <t>01/12/2003</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>IPS (hospital/clínica)</t>
+          <t>Domicilio</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>17/06/2026</t>
+          <t>22/06/2026</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -7472,7 +7472,7 @@
         <v>1</v>
       </c>
       <c r="S58" t="n">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="T58" t="inlineStr">
         <is>
@@ -7486,7 +7486,7 @@
       </c>
       <c r="V58" t="inlineStr">
         <is>
-          <t>O99.3</t>
+          <t>O41.1</t>
         </is>
       </c>
       <c r="W58" t="n">
@@ -7508,7 +7508,7 @@
       </c>
       <c r="AB58" t="inlineStr">
         <is>
-          <t>Ninguna</t>
+          <t>Migrante</t>
         </is>
       </c>
       <c r="AC58" t="inlineStr">
@@ -7538,17 +7538,17 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>10/11/1988</t>
+          <t>19/01/1996</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Otro</t>
+          <t>IPS (hospital/clínica)</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>31/07/2025</t>
+          <t>08/10/2025</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -7594,7 +7594,7 @@
         <v>1</v>
       </c>
       <c r="S59" t="n">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="T59" t="inlineStr">
         <is>
@@ -7608,7 +7608,7 @@
       </c>
       <c r="V59" t="inlineStr">
         <is>
-          <t>O26.6</t>
+          <t>O44.0</t>
         </is>
       </c>
       <c r="W59" t="n">
@@ -7640,7 +7640,7 @@
       </c>
       <c r="AD59" t="inlineStr">
         <is>
-          <t>Contributivo</t>
+          <t>Subsidiado</t>
         </is>
       </c>
     </row>
@@ -7660,17 +7660,17 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>19/11/1994</t>
+          <t>07/12/1983</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>IPS (centro/puesto salud)</t>
+          <t>IPS (centro/puesto de salud)</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>21/03/2026</t>
+          <t>07/04/2025</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -7716,7 +7716,7 @@
         <v>4</v>
       </c>
       <c r="S60" t="n">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="T60" t="inlineStr">
         <is>
@@ -7730,7 +7730,7 @@
       </c>
       <c r="V60" t="inlineStr">
         <is>
-          <t>O44.0</t>
+          <t>O08.1</t>
         </is>
       </c>
       <c r="W60" t="n">
@@ -7752,12 +7752,12 @@
       </c>
       <c r="AB60" t="inlineStr">
         <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="AC60" t="inlineStr">
+        <is>
           <t>Indígena</t>
-        </is>
-      </c>
-      <c r="AC60" t="inlineStr">
-        <is>
-          <t>Ninguna</t>
         </is>
       </c>
       <c r="AD60" t="inlineStr">
@@ -7782,17 +7782,17 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>13/04/1994</t>
+          <t>09/12/1986</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Lugar de trabajo</t>
+          <t>Vía pública</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>11/12/2025</t>
+          <t>08/08/2025</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -7838,7 +7838,7 @@
         <v>2</v>
       </c>
       <c r="S61" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="T61" t="inlineStr">
         <is>
@@ -7852,7 +7852,7 @@
       </c>
       <c r="V61" t="inlineStr">
         <is>
-          <t>O08.1</t>
+          <t>O15.0</t>
         </is>
       </c>
       <c r="W61" t="n">
@@ -7874,7 +7874,7 @@
       </c>
       <c r="AB61" t="inlineStr">
         <is>
-          <t>Discapacidad</t>
+          <t>Ninguna</t>
         </is>
       </c>
       <c r="AC61" t="inlineStr">

</xml_diff>